<commit_message>
cargas 2026: precios de la semana 38 (Fisher 38, Cassio 35, Ivo 43) segun la nota completa de Gonzalo; dias de Paraguay sem 40 confirmados
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -2406,7 +2406,9 @@
       <c r="C29" s="6">
         <v>1</v>
       </c>
-      <c r="D29" s="8"/>
+      <c r="D29" s="8">
+        <v>38</v>
+      </c>
       <c r="E29" s="11" t="s">
         <v>24</v>
       </c>
@@ -2421,7 +2423,9 @@
       <c r="C30" s="6">
         <v>1</v>
       </c>
-      <c r="D30" s="8"/>
+      <c r="D30" s="8">
+        <v>35</v>
+      </c>
       <c r="E30" s="11" t="s">
         <v>34</v>
       </c>
@@ -2436,7 +2440,9 @@
       <c r="C31" s="6">
         <v>1</v>
       </c>
-      <c r="D31" s="8"/>
+      <c r="D31" s="8">
+        <v>43</v>
+      </c>
       <c r="E31" s="11" t="s">
         <v>29</v>
       </c>

</xml_diff>

<commit_message>
resumen WhatsApp: clima una linea por zona con numeros del pronostico, cajas del Plan de Cargas con control de verosimilitud, lectura con la semana primero; precios semana 40 en cargas 2026.xlsx
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -2043,7 +2043,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J91"/>
+  <dimension ref="B2:J92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -2088,7 +2088,7 @@
         <v>18</v>
       </c>
       <c r="J5" s="12">
-        <f>SUM(C21,C36,C54,C73,C91)</f>
+        <f>SUM(C21,C36,C54,C74,C92)</f>
         <v>14.5</v>
       </c>
     </row>
@@ -2112,7 +2112,7 @@
         <v>21</v>
       </c>
       <c r="J6" s="12" t="e">
-        <f>AVERAGE(D21,D36,D54,D73,D91)</f>
+        <f>AVERAGE(D21,D36,D54,D74,D92)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -2693,7 +2693,9 @@
       <c r="C62" s="6">
         <v>1</v>
       </c>
-      <c r="D62" s="8"/>
+      <c r="D62" s="8">
+        <v>36</v>
+      </c>
       <c r="E62" s="11" t="s">
         <v>29</v>
       </c>
@@ -2708,7 +2710,9 @@
       <c r="C63" s="6">
         <v>1</v>
       </c>
-      <c r="D63" s="8"/>
+      <c r="D63" s="8">
+        <v>36</v>
+      </c>
       <c r="E63" s="11" t="s">
         <v>29</v>
       </c>
@@ -2723,7 +2727,9 @@
       <c r="C64" s="6">
         <v>1</v>
       </c>
-      <c r="D64" s="8"/>
+      <c r="D64" s="8">
+        <v>35</v>
+      </c>
       <c r="E64" s="11" t="s">
         <v>24</v>
       </c>
@@ -2733,12 +2739,14 @@
     </row>
     <row r="65">
       <c r="B65" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C65" s="6">
         <v>1</v>
       </c>
-      <c r="D65" s="8"/>
+      <c r="D65" s="8">
+        <v>35</v>
+      </c>
       <c r="E65" s="11" t="s">
         <v>24</v>
       </c>
@@ -2753,7 +2761,9 @@
       <c r="C66" s="6">
         <v>1</v>
       </c>
-      <c r="D66" s="8"/>
+      <c r="D66" s="8">
+        <v>43</v>
+      </c>
       <c r="E66" s="11" t="s">
         <v>27</v>
       </c>
@@ -2768,7 +2778,9 @@
       <c r="C67" s="6">
         <v>1</v>
       </c>
-      <c r="D67" s="8"/>
+      <c r="D67" s="8">
+        <v>43</v>
+      </c>
       <c r="E67" s="11" t="s">
         <v>27</v>
       </c>
@@ -2783,7 +2795,9 @@
       <c r="C68" s="6">
         <v>1</v>
       </c>
-      <c r="D68" s="8"/>
+      <c r="D68" s="8">
+        <v>35</v>
+      </c>
       <c r="E68" s="11" t="s">
         <v>34</v>
       </c>
@@ -2798,7 +2812,9 @@
       <c r="C69" s="6">
         <v>1</v>
       </c>
-      <c r="D69" s="8"/>
+      <c r="D69" s="8">
+        <v>40</v>
+      </c>
       <c r="E69" s="11" t="s">
         <v>24</v>
       </c>
@@ -2813,7 +2829,9 @@
       <c r="C70" s="6">
         <v>1</v>
       </c>
-      <c r="D70" s="8"/>
+      <c r="D70" s="8">
+        <v>43</v>
+      </c>
       <c r="E70" s="11" t="s">
         <v>24</v>
       </c>
@@ -2828,7 +2846,9 @@
       <c r="C71" s="6">
         <v>1</v>
       </c>
-      <c r="D71" s="8"/>
+      <c r="D71" s="8">
+        <v>38</v>
+      </c>
       <c r="E71" s="11" t="s">
         <v>24</v>
       </c>
@@ -2838,75 +2858,83 @@
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="B72" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C72" s="6">
+        <v>1</v>
+      </c>
+      <c r="D72" s="8">
+        <v>38</v>
+      </c>
+      <c r="E72" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F72" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C72" s="6">
-        <v>1</v>
-      </c>
-      <c r="D72" s="8"/>
-      <c r="E72" s="11" t="s">
+      <c r="C73" s="6">
+        <v>1</v>
+      </c>
+      <c r="D73" s="8">
+        <v>38</v>
+      </c>
+      <c r="E73" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F72" s="11" t="s">
+      <c r="F73" s="11" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="B73" s="14" t="s">
+    <row r="74" ht="18" customHeight="1">
+      <c r="B74" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C73" s="18">
-        <f>SUM(C62:C72)</f>
-        <v>0</v>
-      </c>
-      <c r="D73" s="19" t="e">
-        <f>AVERAGE(D62:D72)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E73" s="33"/>
-      <c r="F73" s="34"/>
-    </row>
-    <row r="74" ht="18" customHeight="1"/>
+      <c r="C74" s="18">
+        <f>SUM(C62:C73)</f>
+      </c>
+      <c r="D74" s="19">
+        <f>IFERROR(SUMPRODUCT(C62:C73,D62:D73)/SUM(C62:C73),"")</f>
+      </c>
+      <c r="E74" s="33"/>
+      <c r="F74" s="34"/>
+    </row>
     <row r="75" ht="18" customHeight="1"/>
     <row r="76" ht="18" customHeight="1"/>
-    <row r="77" ht="18" customHeight="1">
-      <c r="C77" s="45" t="s">
+    <row r="77" ht="18" customHeight="1"/>
+    <row r="78" ht="18" customHeight="1">
+      <c r="C78" s="45" t="s">
         <v>137</v>
       </c>
-      <c r="D77" s="45"/>
-      <c r="E77" s="45"/>
-    </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="C78" s="45"/>
       <c r="D78" s="45"/>
       <c r="E78" s="45"/>
     </row>
-    <row r="79" ht="18" customHeight="1"/>
-    <row r="80" ht="18" customHeight="1">
-      <c r="B80" s="5" t="s">
+    <row r="79" ht="18" customHeight="1">
+      <c r="C79" s="45"/>
+      <c r="D79" s="45"/>
+      <c r="E79" s="45"/>
+    </row>
+    <row r="80" ht="18" customHeight="1"/>
+    <row r="81" ht="18" customHeight="1">
+      <c r="B81" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C80" s="5" t="s">
+      <c r="C81" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="D81" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E80" s="5" t="s">
+      <c r="E81" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F80" s="5" t="s">
+      <c r="F81" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="B81" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C81" s="6"/>
-      <c r="D81" s="8"/>
-      <c r="E81" s="11"/>
-      <c r="F81" s="11"/>
     </row>
     <row r="82" ht="18" customHeight="1">
       <c r="B82" s="2" t="s">
@@ -2919,7 +2947,7 @@
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="B83" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C83" s="6"/>
       <c r="D83" s="8"/>
@@ -2935,9 +2963,9 @@
       <c r="E84" s="11"/>
       <c r="F84" s="11"/>
     </row>
-    <row r="85">
+    <row r="85" ht="18" customHeight="1">
       <c r="B85" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C85" s="6"/>
       <c r="D85" s="8"/>
@@ -2955,7 +2983,7 @@
     </row>
     <row r="87">
       <c r="B87" s="2" t="s">
-        <v>106</v>
+        <v>8</v>
       </c>
       <c r="C87" s="6"/>
       <c r="D87" s="8"/>
@@ -2964,7 +2992,7 @@
     </row>
     <row r="88">
       <c r="B88" s="2" t="s">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="8"/>
@@ -2973,38 +3001,46 @@
     </row>
     <row r="89">
       <c r="B89" s="2" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="C89" s="6"/>
       <c r="D89" s="8"/>
       <c r="E89" s="11"/>
       <c r="F89" s="11"/>
     </row>
-    <row r="90" ht="15.75">
+    <row r="90">
       <c r="B90" s="2" t="s">
-        <v>127</v>
+        <v>43</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="8"/>
       <c r="E90" s="11"/>
       <c r="F90" s="11"/>
     </row>
-    <row r="91" ht="19.5">
-      <c r="B91" s="14" t="s">
+    <row r="91" ht="15.75">
+      <c r="B91" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C91" s="6"/>
+      <c r="D91" s="8"/>
+      <c r="E91" s="11"/>
+      <c r="F91" s="11"/>
+    </row>
+    <row r="92" ht="19.5">
+      <c r="B92" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C91" s="18">
-        <f>SUM(C81:C90)</f>
+      <c r="C92" s="18">
+        <f>SUM(C82:C91)</f>
         <v>0</v>
       </c>
-      <c r="D91" s="19" t="e">
-        <f>AVERAGE(D81:D90)</f>
+      <c r="D92" s="19" t="e">
+        <f>AVERAGE(D82:D91)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E91" s="33"/>
-      <c r="F91" s="34"/>
-    </row>
-    <row r="93" ht="18" customHeight="1"/>
+      <c r="E92" s="33"/>
+      <c r="F92" s="34"/>
+    </row>
     <row r="94" ht="18" customHeight="1"/>
     <row r="95" ht="18" customHeight="1"/>
     <row r="96" ht="18" customHeight="1"/>
@@ -3017,12 +3053,13 @@
     <row r="103" ht="18" customHeight="1"/>
     <row r="104" ht="18" customHeight="1"/>
     <row r="105" ht="18" customHeight="1"/>
+    <row r="106" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C77:E77"/>
     <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C79:E79"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C25:E25"/>

</xml_diff>

<commit_message>
cargas 2026.xlsx: precios dictados de las semanas 40 (correcciones) y 41 (nueva), Paraguay USD 7 como texto
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
   <si>
     <t>Semana</t>
   </si>
@@ -495,7 +495,34 @@
     <t/>
   </si>
   <si>
-    <t xml:space="preserve">Semana </t>
+    <t>Paraguay (USD/caja)</t>
+  </si>
+  <si>
+    <t>Paraguay MS</t>
+  </si>
+  <si>
+    <t>7 USD</t>
+  </si>
+  <si>
+    <t>lunes</t>
+  </si>
+  <si>
+    <t>Paraguay DF</t>
+  </si>
+  <si>
+    <t>martes</t>
+  </si>
+  <si>
+    <t>Paraguay AS</t>
+  </si>
+  <si>
+    <t>Semana 41</t>
+  </si>
+  <si>
+    <t>05/10 al 10/10</t>
+  </si>
+  <si>
+    <t>Celso</t>
   </si>
 </sst>
 </file>
@@ -2043,7 +2070,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J92"/>
+  <dimension ref="B2:J103"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -2088,7 +2115,7 @@
         <v>18</v>
       </c>
       <c r="J5" s="12">
-        <f>SUM(C21,C36,C54,C74,C92)</f>
+        <f>SUM(C21,C36,C54,C74,C97)</f>
         <v>14.5</v>
       </c>
     </row>
@@ -2112,7 +2139,7 @@
         <v>21</v>
       </c>
       <c r="J6" s="12" t="e">
-        <f>AVERAGE(D21,D36,D54,D74,D92)</f>
+        <f>AVERAGE(D21,D36,D54,D74,D97)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -2694,7 +2721,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="8">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E62" s="11" t="s">
         <v>29</v>
@@ -2711,7 +2738,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="8">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>29</v>
@@ -2813,7 +2840,7 @@
         <v>1</v>
       </c>
       <c r="D69" s="8">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>24</v>
@@ -2903,163 +2930,354 @@
       <c r="E74" s="33"/>
       <c r="F74" s="34"/>
     </row>
-    <row r="75" ht="18" customHeight="1"/>
-    <row r="76" ht="18" customHeight="1"/>
-    <row r="77" ht="18" customHeight="1"/>
-    <row r="78" ht="18" customHeight="1">
-      <c r="C78" s="45" t="s">
+    <row r="75">
+      <c r="B75" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="D78" s="45"/>
-      <c r="E78" s="45"/>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="C79" s="45"/>
-      <c r="D79" s="45"/>
-      <c r="E79" s="45"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="0">
+        <v>1</v>
+      </c>
+      <c r="D76" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E76" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="C77" s="0">
+        <v>1</v>
+      </c>
+      <c r="D77" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E77" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="C78" s="0">
+        <v>1</v>
+      </c>
+      <c r="D78" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E78" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C79" s="0">
+        <v>1</v>
+      </c>
+      <c r="D79" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E79" s="0" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="80" ht="18" customHeight="1"/>
-    <row r="81" ht="18" customHeight="1">
-      <c r="B81" s="5" t="s">
+    <row r="81" ht="18" customHeight="1"/>
+    <row r="82" ht="18" customHeight="1"/>
+    <row r="83" ht="18" customHeight="1">
+      <c r="C83" s="45" t="s">
+        <v>144</v>
+      </c>
+      <c r="D83" s="45"/>
+      <c r="E83" s="45"/>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="C84" s="45" t="s">
+        <v>145</v>
+      </c>
+      <c r="D84" s="45"/>
+      <c r="E84" s="45"/>
+    </row>
+    <row r="85" ht="18" customHeight="1"/>
+    <row r="86" ht="18" customHeight="1">
+      <c r="B86" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C81" s="5" t="s">
+      <c r="C86" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="D86" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E81" s="5" t="s">
+      <c r="E86" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F81" s="5" t="s">
+      <c r="F86" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="B82" s="2" t="s">
+    <row r="87" ht="18" customHeight="1">
+      <c r="B87" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C82" s="6"/>
-      <c r="D82" s="8"/>
-      <c r="E82" s="11"/>
-      <c r="F82" s="11"/>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="B83" s="2" t="s">
+      <c r="C87" s="6">
+        <v>1</v>
+      </c>
+      <c r="D87" s="8">
+        <v>35</v>
+      </c>
+      <c r="E87" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F87" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="B88" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C83" s="6"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="11"/>
-      <c r="F83" s="11"/>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="B84" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C84" s="6"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="11"/>
-      <c r="F84" s="11"/>
-    </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="B85" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C85" s="6"/>
-      <c r="D85" s="8"/>
-      <c r="E85" s="11"/>
-      <c r="F85" s="11"/>
-    </row>
-    <row r="86">
-      <c r="B86" s="2" t="s">
+      <c r="C88" s="6">
+        <v>1</v>
+      </c>
+      <c r="D88" s="8">
+        <v>35</v>
+      </c>
+      <c r="E88" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F88" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="B89" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C86" s="6"/>
-      <c r="D86" s="8"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="11"/>
-    </row>
-    <row r="87">
-      <c r="B87" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C87" s="6"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="11"/>
-      <c r="F87" s="11"/>
-    </row>
-    <row r="88">
-      <c r="B88" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C88" s="6"/>
-      <c r="D88" s="8"/>
-      <c r="E88" s="11"/>
-      <c r="F88" s="11"/>
-    </row>
-    <row r="89">
-      <c r="B89" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C89" s="6"/>
-      <c r="D89" s="8"/>
-      <c r="E89" s="11"/>
-      <c r="F89" s="11"/>
-    </row>
-    <row r="90">
+      <c r="C89" s="6">
+        <v>1</v>
+      </c>
+      <c r="D89" s="8">
+        <v>36</v>
+      </c>
+      <c r="E89" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F89" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
       <c r="B90" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C90" s="6"/>
-      <c r="D90" s="8"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="11"/>
-    </row>
-    <row r="91" ht="15.75">
+      <c r="C90" s="6">
+        <v>1</v>
+      </c>
+      <c r="D90" s="8">
+        <v>43</v>
+      </c>
+      <c r="E90" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F90" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="91">
       <c r="B91" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C91" s="6"/>
-      <c r="D91" s="8"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="11"/>
-    </row>
-    <row r="92" ht="19.5">
-      <c r="B92" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C91" s="6">
+        <v>1</v>
+      </c>
+      <c r="D91" s="8">
+        <v>43</v>
+      </c>
+      <c r="E91" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F91" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C92" s="6">
+        <v>1</v>
+      </c>
+      <c r="D92" s="8">
+        <v>38</v>
+      </c>
+      <c r="E92" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F92" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" s="6">
+        <v>1</v>
+      </c>
+      <c r="D93" s="8">
+        <v>36</v>
+      </c>
+      <c r="E93" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F93" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C94" s="6">
+        <v>1</v>
+      </c>
+      <c r="D94" s="8">
+        <v>43</v>
+      </c>
+      <c r="E94" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F94" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="2"/>
+      <c r="C95" s="6"/>
+      <c r="D95" s="8"/>
+      <c r="E95" s="11"/>
+      <c r="F95" s="11"/>
+    </row>
+    <row r="96" ht="15.75">
+      <c r="B96" s="2"/>
+      <c r="C96" s="6"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="11"/>
+      <c r="F96" s="11"/>
+    </row>
+    <row r="97" ht="19.5">
+      <c r="B97" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C92" s="18">
-        <f>SUM(C82:C91)</f>
-        <v>0</v>
-      </c>
-      <c r="D92" s="19" t="e">
-        <f>AVERAGE(D82:D91)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E92" s="33"/>
-      <c r="F92" s="34"/>
-    </row>
-    <row r="94" ht="18" customHeight="1"/>
-    <row r="95" ht="18" customHeight="1"/>
-    <row r="96" ht="18" customHeight="1"/>
-    <row r="97" ht="18" customHeight="1"/>
-    <row r="98" ht="18" customHeight="1"/>
-    <row r="99" ht="18" customHeight="1"/>
-    <row r="100" ht="18" customHeight="1"/>
-    <row r="101" ht="18" customHeight="1"/>
-    <row r="102" ht="18" customHeight="1"/>
-    <row r="103" ht="18" customHeight="1"/>
+      <c r="C97" s="18">
+        <f>SUM(C87:C96)</f>
+      </c>
+      <c r="D97" s="19">
+        <f>IFERROR(SUMPRODUCT(C87:C96,D87:D96)/SUM(C87:C96),"")</f>
+      </c>
+      <c r="E97" s="33"/>
+      <c r="F97" s="34"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="B99" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C99" s="0">
+        <v>1</v>
+      </c>
+      <c r="D99" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E99" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="B100" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C100" s="0">
+        <v>1</v>
+      </c>
+      <c r="D100" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E100" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="B101" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="C101" s="0">
+        <v>1</v>
+      </c>
+      <c r="D101" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E101" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1">
+      <c r="B102" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="C102" s="0">
+        <v>1</v>
+      </c>
+      <c r="D102" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E102" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="B103" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C103" s="0">
+        <v>1</v>
+      </c>
+      <c r="D103" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E103" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
     <row r="104" ht="18" customHeight="1"/>
     <row r="105" ht="18" customHeight="1"/>
     <row r="106" ht="18" customHeight="1"/>
+    <row r="107" ht="18" customHeight="1"/>
+    <row r="108" ht="18" customHeight="1"/>
+    <row r="109" ht="18" customHeight="1"/>
+    <row r="110" ht="18" customHeight="1"/>
+    <row r="111" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C84:E84"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C25:E25"/>

</xml_diff>

<commit_message>
planificacion 15/10: precios de las semanas 42 y 43 en cargas 2026.xlsx y cargas de las dos semanas en el plan; sab 24 26.032, falta 1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
   <si>
     <t>Semana</t>
   </si>
@@ -523,6 +523,33 @@
   </si>
   <si>
     <t>Celso</t>
+  </si>
+  <si>
+    <t>Semana 42</t>
+  </si>
+  <si>
+    <t>12/10 al 17/10</t>
+  </si>
+  <si>
+    <t>miercoles</t>
+  </si>
+  <si>
+    <t>Semana 43</t>
+  </si>
+  <si>
+    <t>19/10 al 24/10</t>
+  </si>
+  <si>
+    <t>Muller Fabricio</t>
+  </si>
+  <si>
+    <t>Jaime Zimerman</t>
+  </si>
+  <si>
+    <t>Paraguay GM</t>
+  </si>
+  <si>
+    <t>7,5 USD</t>
   </si>
 </sst>
 </file>
@@ -2070,7 +2097,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J103"/>
+  <dimension ref="A2:J157"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -3267,11 +3294,685 @@
     <row r="104" ht="18" customHeight="1"/>
     <row r="105" ht="18" customHeight="1"/>
     <row r="106" ht="18" customHeight="1"/>
-    <row r="107" ht="18" customHeight="1"/>
-    <row r="108" ht="18" customHeight="1"/>
+    <row r="107" ht="18" customHeight="1">
+      <c r="C107" s="0" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="C108" s="0" t="s">
+        <v>148</v>
+      </c>
+    </row>
     <row r="109" ht="18" customHeight="1"/>
-    <row r="110" ht="18" customHeight="1"/>
-    <row r="111" ht="18" customHeight="1"/>
+    <row r="110" ht="18" customHeight="1">
+      <c r="B110" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C110" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D110" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="E110" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="F110" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="B111" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C111" s="0">
+        <v>1</v>
+      </c>
+      <c r="D111" s="0">
+        <v>35</v>
+      </c>
+      <c r="E111" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F111" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" s="0">
+        <v>1</v>
+      </c>
+      <c r="D112" s="0">
+        <v>35</v>
+      </c>
+      <c r="E112" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F112" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C113" s="0">
+        <v>1</v>
+      </c>
+      <c r="D113" s="0">
+        <v>35</v>
+      </c>
+      <c r="E113" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F113" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" s="0">
+        <v>1</v>
+      </c>
+      <c r="D114" s="0">
+        <v>35</v>
+      </c>
+      <c r="E114" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F114" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C115" s="0">
+        <v>1</v>
+      </c>
+      <c r="D115" s="0">
+        <v>35</v>
+      </c>
+      <c r="E115" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="F115" s="0" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C116" s="0">
+        <v>1</v>
+      </c>
+      <c r="D116" s="0">
+        <v>35</v>
+      </c>
+      <c r="E116" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F116" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C117" s="0">
+        <v>1</v>
+      </c>
+      <c r="D117" s="0">
+        <v>38</v>
+      </c>
+      <c r="E117" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F117" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C118" s="0">
+        <v>1</v>
+      </c>
+      <c r="D118" s="0">
+        <v>38</v>
+      </c>
+      <c r="E118" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F118" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C119" s="0">
+        <v>1</v>
+      </c>
+      <c r="D119" s="0">
+        <v>40</v>
+      </c>
+      <c r="E119" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F119" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C120" s="0">
+        <v>1</v>
+      </c>
+      <c r="D120" s="0">
+        <v>38</v>
+      </c>
+      <c r="E120" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F120" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="C121" s="0">
+        <v>1</v>
+      </c>
+      <c r="D121" s="0">
+        <v>40</v>
+      </c>
+      <c r="E121" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F121" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C122" s="0">
+        <v>1</v>
+      </c>
+      <c r="D122" s="0">
+        <v>38</v>
+      </c>
+      <c r="E122" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F122" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C123" s="0">
+        <v>1</v>
+      </c>
+      <c r="D123" s="0">
+        <v>38</v>
+      </c>
+      <c r="E123" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F123" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="C124" s="0">
+        <v>1</v>
+      </c>
+      <c r="D124" s="0">
+        <v>38</v>
+      </c>
+      <c r="E124" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F124" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C125" s="0">
+        <f>SUM(C111:C124)</f>
+      </c>
+      <c r="D125" s="0">
+        <f>IFERROR(SUMPRODUCT(C111:C124,D111:D124)/SUM(C111:C124),"")</f>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C127" s="0">
+        <v>1</v>
+      </c>
+      <c r="D127" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E127" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C128" s="0">
+        <v>1</v>
+      </c>
+      <c r="D128" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E128" s="0" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132">
+      <c r="C132" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="C133" s="0" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="134"/>
+    <row r="135">
+      <c r="B135" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C135" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D135" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="E135" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="F135" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="B136" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" s="0">
+        <v>1</v>
+      </c>
+      <c r="D136" s="0">
+        <v>35</v>
+      </c>
+      <c r="E136" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F136" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="B137" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C137" s="0">
+        <v>1</v>
+      </c>
+      <c r="D137" s="0">
+        <v>35</v>
+      </c>
+      <c r="E137" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F137" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="B138" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="C138" s="0">
+        <v>1</v>
+      </c>
+      <c r="D138" s="0">
+        <v>38</v>
+      </c>
+      <c r="E138" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F138" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="C139" s="0">
+        <v>1</v>
+      </c>
+      <c r="D139" s="0">
+        <v>38</v>
+      </c>
+      <c r="E139" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F139" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C140" s="0">
+        <v>1</v>
+      </c>
+      <c r="E140" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F140" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C141" s="0">
+        <v>1</v>
+      </c>
+      <c r="E141" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F141" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C142" s="0">
+        <v>1</v>
+      </c>
+      <c r="D142" s="0">
+        <v>35</v>
+      </c>
+      <c r="E142" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="F142" s="0" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C143" s="0">
+        <v>1</v>
+      </c>
+      <c r="D143" s="0">
+        <v>35</v>
+      </c>
+      <c r="E143" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F143" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C144" s="0">
+        <v>1</v>
+      </c>
+      <c r="D144" s="0">
+        <v>35</v>
+      </c>
+      <c r="E144" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F144" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="C145" s="0">
+        <v>1</v>
+      </c>
+      <c r="D145" s="0">
+        <v>38</v>
+      </c>
+      <c r="E145" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F145" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="B146" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C146" s="0">
+        <v>1</v>
+      </c>
+      <c r="D146" s="0">
+        <v>40</v>
+      </c>
+      <c r="E146" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F146" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="B147" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="C147" s="0">
+        <v>1</v>
+      </c>
+      <c r="D147" s="0">
+        <v>38</v>
+      </c>
+      <c r="E147" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="F147" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C148" s="0">
+        <v>1</v>
+      </c>
+      <c r="E148" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F148" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C149" s="0">
+        <v>1</v>
+      </c>
+      <c r="E149" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F149" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C150" s="0">
+        <v>1</v>
+      </c>
+      <c r="D150" s="0">
+        <v>38</v>
+      </c>
+      <c r="E150" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F150" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C151" s="0">
+        <v>1</v>
+      </c>
+      <c r="D151" s="0">
+        <v>38</v>
+      </c>
+      <c r="E151" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F151" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="C152" s="0">
+        <v>1</v>
+      </c>
+      <c r="D152" s="0">
+        <v>38</v>
+      </c>
+      <c r="E152" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F152" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C153" s="0">
+        <v>1</v>
+      </c>
+      <c r="D153" s="0">
+        <v>38</v>
+      </c>
+      <c r="E153" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F153" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C154" s="0">
+        <f>SUM(C136:C153)</f>
+      </c>
+      <c r="D154" s="0">
+        <f>IFERROR(SUMPRODUCT(C136:C153,D136:D153)/SUM(C136:C153),"")</f>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C156" s="0">
+        <v>1</v>
+      </c>
+      <c r="D156" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E156" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="C157" s="0">
+        <v>1</v>
+      </c>
+      <c r="D157" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="E157" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="C58:E58"/>

</xml_diff>

<commit_message>
plan de compras: BAHIA vie 23 y Sergio Correia sab 24 (descargan la semana del 26); precios en la semana 43
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t>Semana</t>
   </si>
@@ -544,6 +544,12 @@
   </si>
   <si>
     <t>Jaime Zimerman</t>
+  </si>
+  <si>
+    <t>BAHIA</t>
+  </si>
+  <si>
+    <t>Sergio Correia</t>
   </si>
   <si>
     <t>Paraguay GM</t>
@@ -2097,7 +2103,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="A2:J157"/>
+  <dimension ref="B2:J159"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -3604,9 +3610,6 @@
         <v>149</v>
       </c>
     </row>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
     <row r="132">
       <c r="C132" s="0" t="s">
         <v>150</v>
@@ -3617,7 +3620,6 @@
         <v>151</v>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="B135" s="0" t="s">
         <v>2</v>
@@ -3931,45 +3933,70 @@
     </row>
     <row r="154">
       <c r="B154" s="0" t="s">
-        <v>13</v>
+        <v>154</v>
       </c>
       <c r="C154" s="0">
-        <f>SUM(C136:C153)</f>
+        <v>1</v>
       </c>
       <c r="D154" s="0">
-        <f>IFERROR(SUMPRODUCT(C136:C153,D136:D153)/SUM(C136:C153),"")</f>
+        <v>38</v>
+      </c>
+      <c r="E154" s="0" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="155">
       <c r="B155" s="0" t="s">
-        <v>137</v>
+        <v>155</v>
+      </c>
+      <c r="C155" s="0">
+        <v>1</v>
+      </c>
+      <c r="D155" s="0">
+        <v>36</v>
       </c>
     </row>
     <row r="156">
       <c r="B156" s="0" t="s">
-        <v>138</v>
+        <v>13</v>
       </c>
       <c r="C156" s="0">
-        <v>1</v>
-      </c>
-      <c r="D156" s="0" t="s">
-        <v>139</v>
-      </c>
-      <c r="E156" s="0" t="s">
-        <v>140</v>
+        <f>SUM(C136:C155)</f>
+      </c>
+      <c r="D156" s="0">
+        <f>IFERROR(SUMPRODUCT(C136:C155,D136:D155)/SUM(C136:C155),"")</f>
       </c>
     </row>
     <row r="157">
       <c r="B157" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="C157" s="0">
-        <v>1</v>
-      </c>
-      <c r="D157" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="E157" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C158" s="0">
+        <v>1</v>
+      </c>
+      <c r="D158" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E158" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="C159" s="0">
+        <v>1</v>
+      </c>
+      <c r="D159" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="E159" s="0" t="s">
         <v>140</v>
       </c>
     </row>

</xml_diff>

<commit_message>
plan de compras: dictado definitivo semana 19-25/10 con precios; Semana 43 de cargas 2026.xlsx rehecha
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>Semana</t>
   </si>
@@ -538,18 +538,6 @@
   </si>
   <si>
     <t>19/10 al 24/10</t>
-  </si>
-  <si>
-    <t>Muller Fabricio</t>
-  </si>
-  <si>
-    <t>Jaime Zimerman</t>
-  </si>
-  <si>
-    <t>BAHIA</t>
-  </si>
-  <si>
-    <t>Sergio Correia</t>
   </si>
   <si>
     <t>Paraguay GM</t>
@@ -2103,7 +2091,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J159"/>
+  <dimension ref="B2:J138"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -3639,36 +3627,18 @@
     </row>
     <row r="136">
       <c r="B136" s="0" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C136" s="0">
-        <v>1</v>
+        <f>SUM(C136:C135)</f>
       </c>
       <c r="D136" s="0">
-        <v>35</v>
-      </c>
-      <c r="E136" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="F136" s="0" t="s">
-        <v>23</v>
+        <f>IFERROR(SUMPRODUCT(C136:C135,D136:D135)/SUM(C136:C135),"")</f>
       </c>
     </row>
     <row r="137">
       <c r="B137" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C137" s="0">
-        <v>1</v>
-      </c>
-      <c r="D137" s="0">
-        <v>35</v>
-      </c>
-      <c r="E137" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="F137" s="0" t="s">
-        <v>23</v>
+        <v>137</v>
       </c>
     </row>
     <row r="138">
@@ -3678,325 +3648,10 @@
       <c r="C138" s="0">
         <v>1</v>
       </c>
-      <c r="D138" s="0">
-        <v>38</v>
+      <c r="D138" s="0" t="s">
+        <v>153</v>
       </c>
       <c r="E138" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="F138" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="B139" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="C139" s="0">
-        <v>1</v>
-      </c>
-      <c r="D139" s="0">
-        <v>38</v>
-      </c>
-      <c r="E139" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="F139" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="B140" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="C140" s="0">
-        <v>1</v>
-      </c>
-      <c r="E140" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="F140" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="B141" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="C141" s="0">
-        <v>1</v>
-      </c>
-      <c r="E141" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="F141" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="B142" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="C142" s="0">
-        <v>1</v>
-      </c>
-      <c r="D142" s="0">
-        <v>35</v>
-      </c>
-      <c r="E142" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="F142" s="0" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="B143" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="C143" s="0">
-        <v>1</v>
-      </c>
-      <c r="D143" s="0">
-        <v>35</v>
-      </c>
-      <c r="E143" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F143" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="B144" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="C144" s="0">
-        <v>1</v>
-      </c>
-      <c r="D144" s="0">
-        <v>35</v>
-      </c>
-      <c r="E144" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F144" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="B145" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="C145" s="0">
-        <v>1</v>
-      </c>
-      <c r="D145" s="0">
-        <v>38</v>
-      </c>
-      <c r="E145" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F145" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="B146" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="C146" s="0">
-        <v>1</v>
-      </c>
-      <c r="D146" s="0">
-        <v>40</v>
-      </c>
-      <c r="E146" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F146" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="B147" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="C147" s="0">
-        <v>1</v>
-      </c>
-      <c r="D147" s="0">
-        <v>38</v>
-      </c>
-      <c r="E147" s="0" t="s">
-        <v>136</v>
-      </c>
-      <c r="F147" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="B148" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="C148" s="0">
-        <v>1</v>
-      </c>
-      <c r="E148" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F148" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="B149" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="C149" s="0">
-        <v>1</v>
-      </c>
-      <c r="E149" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F149" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="B150" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C150" s="0">
-        <v>1</v>
-      </c>
-      <c r="D150" s="0">
-        <v>38</v>
-      </c>
-      <c r="E150" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F150" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="B151" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C151" s="0">
-        <v>1</v>
-      </c>
-      <c r="D151" s="0">
-        <v>38</v>
-      </c>
-      <c r="E151" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F151" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="B152" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="C152" s="0">
-        <v>1</v>
-      </c>
-      <c r="D152" s="0">
-        <v>38</v>
-      </c>
-      <c r="E152" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F152" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="B153" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="C153" s="0">
-        <v>1</v>
-      </c>
-      <c r="D153" s="0">
-        <v>38</v>
-      </c>
-      <c r="E153" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F153" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="B154" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="C154" s="0">
-        <v>1</v>
-      </c>
-      <c r="D154" s="0">
-        <v>38</v>
-      </c>
-      <c r="E154" s="0" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="B155" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="C155" s="0">
-        <v>1</v>
-      </c>
-      <c r="D155" s="0">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="B156" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="C156" s="0">
-        <f>SUM(C136:C155)</f>
-      </c>
-      <c r="D156" s="0">
-        <f>IFERROR(SUMPRODUCT(C136:C155,D136:D155)/SUM(C136:C155),"")</f>
-      </c>
-    </row>
-    <row r="157">
-      <c r="B157" s="0" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="C158" s="0">
-        <v>1</v>
-      </c>
-      <c r="D158" s="0" t="s">
-        <v>139</v>
-      </c>
-      <c r="E158" s="0" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="B159" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C159" s="0">
-        <v>1</v>
-      </c>
-      <c r="D159" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="E159" s="0" t="s">
         <v>140</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cargas 2026.xlsx: precios de la Semana 43 (23 BR + Guido) del dictado definitivo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t>Semana</t>
   </si>
@@ -538,6 +538,18 @@
   </si>
   <si>
     <t>19/10 al 24/10</t>
+  </si>
+  <si>
+    <t>Muller Fabricio</t>
+  </si>
+  <si>
+    <t>BAHIA</t>
+  </si>
+  <si>
+    <t>Jhony Viera</t>
+  </si>
+  <si>
+    <t>Jaime Zimerman</t>
   </si>
   <si>
     <t>Paraguay GM</t>
@@ -2091,7 +2103,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J138"/>
+  <dimension ref="B2:J161"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -3627,18 +3639,36 @@
     </row>
     <row r="136">
       <c r="B136" s="0" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C136" s="0">
-        <f>SUM(C136:C135)</f>
+        <v>1</v>
       </c>
       <c r="D136" s="0">
-        <f>IFERROR(SUMPRODUCT(C136:C135,D136:D135)/SUM(C136:C135),"")</f>
+        <v>35</v>
+      </c>
+      <c r="E136" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F136" s="0" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="137">
       <c r="B137" s="0" t="s">
-        <v>137</v>
+        <v>9</v>
+      </c>
+      <c r="C137" s="0">
+        <v>1</v>
+      </c>
+      <c r="D137" s="0">
+        <v>35</v>
+      </c>
+      <c r="E137" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F137" s="0" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="138">
@@ -3648,10 +3678,383 @@
       <c r="C138" s="0">
         <v>1</v>
       </c>
-      <c r="D138" s="0" t="s">
+      <c r="D138" s="0">
+        <v>38</v>
+      </c>
+      <c r="E138" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F138" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="C139" s="0">
+        <v>1</v>
+      </c>
+      <c r="D139" s="0">
+        <v>38</v>
+      </c>
+      <c r="E139" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F139" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="C140" s="0">
+        <v>1</v>
+      </c>
+      <c r="D140" s="0">
+        <v>38</v>
+      </c>
+      <c r="E140" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F140" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C141" s="0">
+        <v>1</v>
+      </c>
+      <c r="D141" s="0">
+        <v>38</v>
+      </c>
+      <c r="E141" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F141" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C142" s="0">
+        <v>1</v>
+      </c>
+      <c r="D142" s="0">
+        <v>38</v>
+      </c>
+      <c r="E142" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F142" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C143" s="0">
+        <v>1</v>
+      </c>
+      <c r="D143" s="0">
+        <v>38</v>
+      </c>
+      <c r="E143" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F143" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="E138" s="0" t="s">
+      <c r="C144" s="0">
+        <v>1</v>
+      </c>
+      <c r="D144" s="0">
+        <v>38</v>
+      </c>
+      <c r="E144" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="F144" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C145" s="0">
+        <v>1</v>
+      </c>
+      <c r="D145" s="0">
+        <v>36</v>
+      </c>
+      <c r="E145" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F145" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="B146" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C146" s="0">
+        <v>1</v>
+      </c>
+      <c r="D146" s="0">
+        <v>35</v>
+      </c>
+      <c r="E146" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="F146" s="0" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="B147" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C147" s="0">
+        <v>1</v>
+      </c>
+      <c r="D147" s="0">
+        <v>35</v>
+      </c>
+      <c r="E147" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F147" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C148" s="0">
+        <v>1</v>
+      </c>
+      <c r="D148" s="0">
+        <v>35</v>
+      </c>
+      <c r="E148" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F148" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="C149" s="0">
+        <v>1</v>
+      </c>
+      <c r="D149" s="0">
+        <v>38</v>
+      </c>
+      <c r="E149" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F149" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="C150" s="0">
+        <v>1</v>
+      </c>
+      <c r="D150" s="0">
+        <v>38</v>
+      </c>
+      <c r="E150" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F150" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C151" s="0">
+        <v>1</v>
+      </c>
+      <c r="D151" s="0">
+        <v>38</v>
+      </c>
+      <c r="E151" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F151" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="C152" s="0">
+        <v>1</v>
+      </c>
+      <c r="D152" s="0">
+        <v>38</v>
+      </c>
+      <c r="E152" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F152" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C153" s="0">
+        <v>1</v>
+      </c>
+      <c r="D153" s="0">
+        <v>35</v>
+      </c>
+      <c r="E153" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F153" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C154" s="0">
+        <v>1</v>
+      </c>
+      <c r="D154" s="0">
+        <v>35</v>
+      </c>
+      <c r="E154" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F154" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C155" s="0">
+        <v>1</v>
+      </c>
+      <c r="D155" s="0">
+        <v>38</v>
+      </c>
+      <c r="E155" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F155" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C156" s="0">
+        <v>1</v>
+      </c>
+      <c r="D156" s="0">
+        <v>38</v>
+      </c>
+      <c r="E156" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F156" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="C157" s="0">
+        <v>1</v>
+      </c>
+      <c r="D157" s="0">
+        <v>38</v>
+      </c>
+      <c r="E157" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F157" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C158" s="0">
+        <v>1</v>
+      </c>
+      <c r="D158" s="0">
+        <v>38</v>
+      </c>
+      <c r="E158" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F158" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C159" s="0">
+        <f>SUM(C136:C158)</f>
+      </c>
+      <c r="D159" s="0">
+        <f>IFERROR(SUMPRODUCT(C136:C158,D136:D158)/SUM(C136:C158),"")</f>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="C161" s="0">
+        <v>1</v>
+      </c>
+      <c r="D161" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="E161" s="0" t="s">
         <v>140</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cargas 2026.xlsx: precios de la semana 44 (26-31/10)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t>Semana</t>
   </si>
@@ -556,6 +556,18 @@
   </si>
   <si>
     <t>7,5 USD</t>
+  </si>
+  <si>
+    <t>Semana 44</t>
+  </si>
+  <si>
+    <t>26/10 al 31/10</t>
+  </si>
+  <si>
+    <t>Andre Pauli</t>
+  </si>
+  <si>
+    <t>Aryste Mittelman</t>
   </si>
 </sst>
 </file>
@@ -2103,7 +2115,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J161"/>
+  <dimension ref="B2:J185"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -4056,6 +4068,268 @@
       </c>
       <c r="E161" s="0" t="s">
         <v>140</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="C165" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="C166" s="0" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="B168" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C168" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D168" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="E168" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="F168" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C169" s="0">
+        <v>1</v>
+      </c>
+      <c r="D169" s="0">
+        <v>31</v>
+      </c>
+      <c r="E169" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C170" s="0">
+        <v>1</v>
+      </c>
+      <c r="D170" s="0">
+        <v>31</v>
+      </c>
+      <c r="E170" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C171" s="0">
+        <v>1</v>
+      </c>
+      <c r="D171" s="0">
+        <v>31</v>
+      </c>
+      <c r="E171" s="0" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C172" s="0">
+        <v>1</v>
+      </c>
+      <c r="D172" s="0">
+        <v>31</v>
+      </c>
+      <c r="E172" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C173" s="0">
+        <v>1</v>
+      </c>
+      <c r="D173" s="0">
+        <v>33</v>
+      </c>
+      <c r="E173" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C174" s="0">
+        <v>1</v>
+      </c>
+      <c r="D174" s="0">
+        <v>32</v>
+      </c>
+      <c r="E174" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="B175" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="C175" s="0">
+        <v>1</v>
+      </c>
+      <c r="D175" s="0">
+        <v>33</v>
+      </c>
+      <c r="E175" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="C176" s="0">
+        <v>1</v>
+      </c>
+      <c r="D176" s="0">
+        <v>33</v>
+      </c>
+      <c r="E176" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="B177" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="C177" s="0">
+        <v>1</v>
+      </c>
+      <c r="D177" s="0">
+        <v>38</v>
+      </c>
+      <c r="E177" s="0" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="C178" s="0">
+        <v>1</v>
+      </c>
+      <c r="D178" s="0">
+        <v>33</v>
+      </c>
+      <c r="E178" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="B179" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C179" s="0">
+        <v>1</v>
+      </c>
+      <c r="D179" s="0">
+        <v>33</v>
+      </c>
+      <c r="E179" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="B180" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C180" s="0">
+        <v>1</v>
+      </c>
+      <c r="D180" s="0">
+        <v>34</v>
+      </c>
+      <c r="E180" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="B181" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="C181" s="0">
+        <v>1</v>
+      </c>
+      <c r="D181" s="0">
+        <v>33</v>
+      </c>
+      <c r="E181" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="B182" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="C182" s="0">
+        <v>1</v>
+      </c>
+      <c r="D182" s="0">
+        <v>33</v>
+      </c>
+      <c r="E182" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="B183" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C183" s="0">
+        <v>1</v>
+      </c>
+      <c r="D183" s="0">
+        <v>33</v>
+      </c>
+      <c r="E183" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="B184" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="C184" s="0">
+        <v>1</v>
+      </c>
+      <c r="D184" s="0">
+        <v>33</v>
+      </c>
+      <c r="E184" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="B185" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C185" s="0">
+        <f>SUM(C169:C184)</f>
+      </c>
+      <c r="D185" s="0">
+        <f>IFERROR(SUMPRODUCT(C169:C184,D169:D184)/SUM(C169:C184),"")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cargas 2026.xlsx: Semana 44 con Cassio del sabado 31 (R$ 31) y Paraguay a 8 USD (el commit anterior solo llevo la nota del README)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/cargas 2026.xlsx
+++ b/fuentes/cargas 2026.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t>Semana</t>
   </si>
@@ -568,6 +568,9 @@
   </si>
   <si>
     <t>Aryste Mittelman</t>
+  </si>
+  <si>
+    <t>8 USD</t>
   </si>
 </sst>
 </file>
@@ -2115,7 +2118,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1258FB-3560-4958-9517-8E4782DDD67C}">
-  <dimension ref="B2:J185"/>
+  <dimension ref="B2:J189"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -4323,13 +4326,57 @@
     </row>
     <row r="185">
       <c r="B185" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C185" s="0">
+        <v>1</v>
+      </c>
+      <c r="D185" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C185" s="0">
-        <f>SUM(C169:C184)</f>
-      </c>
-      <c r="D185" s="0">
-        <f>IFERROR(SUMPRODUCT(C169:C184,D169:D184)/SUM(C169:C184),"")</f>
+      <c r="C186" s="0">
+        <f>SUM(C169:C185)</f>
+      </c>
+      <c r="D186" s="0">
+        <f>IFERROR(SUMPRODUCT(C169:C185,D169:D185)/SUM(C169:C185),"")</f>
+      </c>
+    </row>
+    <row r="187">
+      <c r="B187" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="B188" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C188" s="0">
+        <v>1</v>
+      </c>
+      <c r="D188" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="E188" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C189" s="0">
+        <v>1</v>
+      </c>
+      <c r="D189" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="E189" s="0" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -5847,7 +5894,7 @@
       </c>
       <c r="I6" s="12">
         <f>AVERAGE(D20,D41,D61,D82)</f>
-        <v>36.17628205128206</v>
+        <v>36.176282051282058</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -6959,7 +7006,7 @@
       </c>
       <c r="J6" s="12">
         <f>AVERAGE(D45,D22,D72,D99)</f>
-        <v>52.87730263157895</v>
+        <v>52.877302631578949</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -7903,7 +7950,7 @@
       </c>
       <c r="D72" s="19">
         <f>AVERAGE(D53:D71)</f>
-        <v>58.36842105263158</v>
+        <v>58.368421052631582</v>
       </c>
       <c r="E72" s="35">
         <v>1.92</v>
@@ -8276,7 +8323,7 @@
       </c>
       <c r="D99" s="19">
         <f>AVERAGE(D80:D98)</f>
-        <v>53.31578947368421</v>
+        <v>53.315789473684212</v>
       </c>
       <c r="E99" s="35">
         <v>1.89</v>
@@ -11017,7 +11064,7 @@
       </c>
       <c r="D19" s="19">
         <f>AVERAGE(D6:D18)</f>
-        <v>34.76923076923077</v>
+        <v>34.769230769230766</v>
       </c>
       <c r="E19" s="33"/>
       <c r="F19" s="34"/>
@@ -11278,7 +11325,7 @@
       </c>
       <c r="D40" s="19">
         <f>AVERAGE(D27:D39)</f>
-        <v>37.69230769230769</v>
+        <v>37.692307692307693</v>
       </c>
       <c r="E40" s="33"/>
       <c r="F40" s="34"/>
@@ -11545,7 +11592,7 @@
       </c>
       <c r="D61" s="19">
         <f>AVERAGE(D48:D60)</f>
-        <v>42.61538461538461</v>
+        <v>42.615384615384613</v>
       </c>
       <c r="E61" s="35"/>
       <c r="F61" s="36"/>
@@ -12480,7 +12527,7 @@
       </c>
       <c r="D51" s="19">
         <f>AVERAGE(D40:D50)</f>
-        <v>42.54545454545455</v>
+        <v>42.545454545454547</v>
       </c>
       <c r="E51" s="33"/>
       <c r="F51" s="34"/>
@@ -12924,7 +12971,7 @@
       </c>
       <c r="J6" s="12">
         <f>AVERAGE(D14,D29,D47,D66,D84)</f>
-        <v>40.88298701298701</v>
+        <v>40.882987012987009</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -13222,7 +13269,7 @@
       </c>
       <c r="D29" s="19">
         <f>AVERAGE(D22:D28)</f>
-        <v>44.42857142857143</v>
+        <v>44.428571428571431</v>
       </c>
       <c r="E29" s="33"/>
       <c r="F29" s="34"/>
@@ -13679,7 +13726,7 @@
       </c>
       <c r="D66" s="19">
         <f>AVERAGE(D55:D65)</f>
-        <v>37.63636363636363</v>
+        <v>37.636363636363633</v>
       </c>
       <c r="E66" s="33"/>
       <c r="F66" s="34"/>

</xml_diff>